<commit_message>
Add refined data files to Repo and IPSL-extended ScenarioMIP files
</commit_message>
<xml_diff>
--- a/Data/OHC_diff_totals_output_glob.xlsx
+++ b/Data/OHC_diff_totals_output_glob.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harry\01.HarryGrosvenor\02.Research\05.Local_Repos\202404_01.PlioMIP2_ThetaO\Data\01.thetao\01.OneTime\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCB1CBD-EAFE-4482-AA1F-92397CB15C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D335E4-8D19-4A1D-A562-18F993A836C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9000" yWindow="12852" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -107,8 +107,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000E+00"/>
+    <numFmt numFmtId="165" formatCode="0.0000E+00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -147,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -155,6 +156,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -793,7 +795,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -830,20 +832,20 @@
         <v>4</v>
       </c>
       <c r="B2" s="3">
-        <v>2.186572126346783E+17</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1.516067258405125E+24</v>
+        <v>2.3989053781938909E+17</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1.6597747785739491E+24</v>
       </c>
       <c r="D2" s="3">
-        <v>6933534.1841117106</v>
-      </c>
-      <c r="E2" s="3">
-        <v>2.2010723608654509E+17</v>
-      </c>
-      <c r="F2" s="3">
+        <v>6918883.8945518332</v>
+      </c>
+      <c r="E2">
+        <v>2.4138008611807322E+17</v>
+      </c>
+      <c r="F2" s="7">
         <f>D2*E2</f>
-        <v>1.5261210455764071E+24</v>
+        <v>1.6700807903078712E+24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -851,20 +853,20 @@
         <v>5</v>
       </c>
       <c r="B3" s="3">
-        <v>2.1149832392177651E+17</v>
-      </c>
-      <c r="C3" s="1">
-        <v>2.7498999019900549E+24</v>
+        <v>2.323534923813184E+17</v>
+      </c>
+      <c r="C3" s="3">
+        <v>3.038830534545608E+24</v>
       </c>
       <c r="D3" s="3">
-        <v>13001993.826708131</v>
-      </c>
-      <c r="E3" s="3">
-        <v>2.1490496938728358E+17</v>
-      </c>
-      <c r="F3" s="3">
+        <v>13078480.135596771</v>
+      </c>
+      <c r="E3">
+        <v>2.3603117294852518E+17</v>
+      </c>
+      <c r="F3" s="7">
         <f t="shared" ref="F3:F14" si="0">D3*E3</f>
-        <v>2.7941930853023608E+24</v>
+        <v>3.0869290067888927E+24</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -872,20 +874,20 @@
         <v>6</v>
       </c>
       <c r="B4" s="3">
-        <v>2.186572126346783E+17</v>
-      </c>
-      <c r="C4" s="1">
-        <v>2.310525122032964E+24</v>
+        <v>2.3989053781938909E+17</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2.5343233403141159E+24</v>
       </c>
       <c r="D4" s="3">
-        <v>10566882.7210986</v>
-      </c>
-      <c r="E4" s="3">
-        <v>2.2010723608654509E+17</v>
-      </c>
-      <c r="F4" s="3">
-        <f t="shared" si="0"/>
-        <v>2.3258473497916836E+24</v>
+        <v>10564498.972536299</v>
+      </c>
+      <c r="E4">
+        <v>2.4138008611807322E+17</v>
+      </c>
+      <c r="F4" s="7">
+        <f t="shared" si="0"/>
+        <v>2.5500596717851081E+24</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -893,20 +895,20 @@
         <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>2.1857413248659811E+17</v>
-      </c>
-      <c r="C5" s="1">
-        <v>2.5369149273636799E+24</v>
+        <v>2.3980392349821709E+17</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.7873187196668302E+24</v>
       </c>
       <c r="D5" s="3">
-        <v>11606656.737019099</v>
-      </c>
-      <c r="E5" s="3">
-        <v>2.200902706992264E+17</v>
-      </c>
-      <c r="F5" s="3">
-        <f t="shared" si="0"/>
-        <v>2.5545122231635331E+24</v>
+        <v>11623324.084968749</v>
+      </c>
+      <c r="E5">
+        <v>2.413631143030385E+17</v>
+      </c>
+      <c r="F5" s="7">
+        <f t="shared" si="0"/>
+        <v>2.8054416997015724E+24</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -914,20 +916,20 @@
         <v>8</v>
       </c>
       <c r="B6" s="3">
-        <v>2.186830852014977E+17</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1.6102250868898769E+24</v>
+        <v>2.501195883812497E+17</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1.817861603893894E+24</v>
       </c>
       <c r="D6" s="3">
-        <v>7363281.3685895829</v>
-      </c>
-      <c r="E6" s="3">
-        <v>2.241219067266328E+17</v>
-      </c>
-      <c r="F6" s="3">
-        <f t="shared" si="0"/>
-        <v>1.6502726600929877E+24</v>
+        <v>7267969.7566229142</v>
+      </c>
+      <c r="E6">
+        <v>2.5614027293643021E+17</v>
+      </c>
+      <c r="F6" s="7">
+        <f t="shared" si="0"/>
+        <v>1.8616197571551136E+24</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -935,20 +937,20 @@
         <v>9</v>
       </c>
       <c r="B7" s="3">
-        <v>2.1078733788734141E+17</v>
-      </c>
-      <c r="C7" s="1">
-        <v>2.0064379454873259E+24</v>
+        <v>2.322173544007176E+17</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2.1674058083154629E+24</v>
       </c>
       <c r="D7" s="3">
-        <v>9518778.3364847954</v>
-      </c>
-      <c r="E7" s="3">
-        <v>2.1420200775137581E+17</v>
-      </c>
-      <c r="F7" s="3">
-        <f t="shared" si="0"/>
-        <v>2.0389414310153443E+24</v>
+        <v>9333522.0957489517</v>
+      </c>
+      <c r="E7">
+        <v>2.359043435805791E+17</v>
+      </c>
+      <c r="F7" s="7">
+        <f t="shared" si="0"/>
+        <v>2.2018184032924875E+24</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -956,20 +958,20 @@
         <v>10</v>
       </c>
       <c r="B8" s="3">
-        <v>2.002137228435911E+17</v>
-      </c>
-      <c r="C8" s="1">
-        <v>9.0610466793530355E+23</v>
+        <v>2.364174853728487E+17</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1.048207342601627E+24</v>
       </c>
       <c r="D8" s="3">
-        <v>4525687.1260675834</v>
-      </c>
-      <c r="E8" s="3">
-        <v>2.02489328454712E+17</v>
-      </c>
-      <c r="F8" s="3">
-        <f t="shared" si="0"/>
-        <v>9.1640334695356053E+23</v>
+        <v>4433713.2718780199</v>
+      </c>
+      <c r="E8">
+        <v>2.3890710084718499E+17</v>
+      </c>
+      <c r="F8" s="7">
+        <f t="shared" si="0"/>
+        <v>1.0592455837720646E+24</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -977,20 +979,20 @@
         <v>11</v>
       </c>
       <c r="B9" s="3">
-        <v>1.631988628645287E+17</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1.178690657965942E+24</v>
+        <v>2.2468012852853741E+17</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1.6393661469034719E+24</v>
       </c>
       <c r="D9" s="3">
-        <v>7222419.5516875172</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1.6546850295616131E+17</v>
-      </c>
-      <c r="F9" s="3">
+        <v>7296444.7618929055</v>
+      </c>
+      <c r="E9">
+        <v>2.2714360163890259E+17</v>
+      </c>
+      <c r="F9" s="7">
         <f>D9*E9</f>
-        <v>1.1950829509390431E+24</v>
+        <v>1.6573407423756596E+24</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -998,20 +1000,20 @@
         <v>12</v>
       </c>
       <c r="B10" s="3">
-        <v>2.189660953134705E+17</v>
-      </c>
-      <c r="C10" s="1">
-        <v>2.779834778076861E+24</v>
+        <v>2.4067566257426051E+17</v>
+      </c>
+      <c r="C10" s="3">
+        <v>3.0379232427261271E+24</v>
       </c>
       <c r="D10" s="3">
-        <v>12695274.91960464</v>
-      </c>
-      <c r="E10" s="3">
-        <v>2.189660953134705E+17</v>
-      </c>
-      <c r="F10" s="3">
-        <f t="shared" si="0"/>
-        <v>2.779834778076861E+24</v>
+        <v>12622477.94493461</v>
+      </c>
+      <c r="E10">
+        <v>2.4067566257426051E+17</v>
+      </c>
+      <c r="F10" s="7">
+        <f t="shared" si="0"/>
+        <v>3.0379232427261277E+24</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1019,20 +1021,20 @@
         <v>13</v>
       </c>
       <c r="B11" s="3">
-        <v>2.1286690376051411E+17</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1.3840598669706119E+24</v>
+        <v>2.3445306888129229E+17</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1.5269866982621891E+24</v>
       </c>
       <c r="D11" s="3">
-        <v>6501996.5176350204</v>
-      </c>
-      <c r="E11" s="3">
-        <v>2.1314710896253549E+17</v>
-      </c>
-      <c r="F11" s="3">
-        <f t="shared" si="0"/>
-        <v>1.3858817602183779E+24</v>
+        <v>6512973.8141125739</v>
+      </c>
+      <c r="E11">
+        <v>2.3473445781112122E+17</v>
+      </c>
+      <c r="F11" s="7">
+        <f t="shared" si="0"/>
+        <v>1.5288193769937453E+24</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1040,20 +1042,20 @@
         <v>14</v>
       </c>
       <c r="B12" s="3">
-        <v>1.9767394294476109E+17</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1.3904318142481091E+24</v>
+        <v>2.3531353702562099E+17</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1.6635294314418069E+24</v>
       </c>
       <c r="D12" s="3">
-        <v>7033966.103649064</v>
-      </c>
-      <c r="E12" s="3">
-        <v>2.001721941340833E+17</v>
-      </c>
-      <c r="F12" s="3">
-        <f t="shared" si="0"/>
-        <v>1.4080044284322019E+24</v>
+        <v>7069416.627997403</v>
+      </c>
+      <c r="E12">
+        <v>2.3812234245352371E+17</v>
+      </c>
+      <c r="F12" s="7">
+        <f t="shared" si="0"/>
+        <v>1.6833860472386325E+24</v>
       </c>
       <c r="H12" s="3"/>
     </row>
@@ -1062,20 +1064,20 @@
         <v>15</v>
       </c>
       <c r="B13" s="3">
-        <v>2.1081051174148771E+17</v>
-      </c>
-      <c r="C13" s="1">
-        <v>1.097023898426961E+24</v>
+        <v>2.2639264303773469E+17</v>
+      </c>
+      <c r="C13" s="3">
+        <v>1.175326697778544E+24</v>
       </c>
       <c r="D13" s="3">
-        <v>5203838.6955400854</v>
-      </c>
-      <c r="E13" s="3">
-        <v>2.1088286808967101E+17</v>
-      </c>
-      <c r="F13" s="3">
-        <f t="shared" si="0"/>
-        <v>1.0974004291915055E+24</v>
+        <v>5191541.0412989566</v>
+      </c>
+      <c r="E13">
+        <v>2.2646499938591802E+17</v>
+      </c>
+      <c r="F13" s="7">
+        <f t="shared" si="0"/>
+        <v>1.1757023387297364E+24</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1083,20 +1085,20 @@
         <v>16</v>
       </c>
       <c r="B14" s="3">
-        <v>2.1711973694236941E+17</v>
-      </c>
-      <c r="C14" s="1">
-        <v>9.8754511794162196E+23</v>
+        <v>2.3312039415470211E+17</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1.059632857178943E+24</v>
       </c>
       <c r="D14" s="3">
-        <v>4548389.4363954039</v>
-      </c>
-      <c r="E14" s="3">
-        <v>2.171921624912152E+17</v>
-      </c>
-      <c r="F14" s="3">
-        <f t="shared" si="0"/>
-        <v>9.8787453754291724E+23</v>
+        <v>4545431.818701175</v>
+      </c>
+      <c r="E14">
+        <v>2.33192819703548E+17</v>
+      </c>
+      <c r="F14" s="7">
+        <f t="shared" si="0"/>
+        <v>1.0599620625731534E+24</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1105,23 +1107,23 @@
       </c>
       <c r="B15" s="4">
         <f>AVERAGE(B2:B14)</f>
-        <v>2.0905439085979174E+17</v>
+        <v>2.3579448875963677E+17</v>
       </c>
       <c r="C15" s="4">
         <f>AVERAGE(C2:C14)</f>
-        <v>1.7272123879795722E+24</v>
+        <v>1.9351144001694285E+24</v>
       </c>
       <c r="D15" s="4">
         <f>AVERAGE(D2:D14)</f>
-        <v>8209438.4249685565</v>
+        <v>8189129.093910858</v>
       </c>
       <c r="E15" s="4">
         <f>AVERAGE(E2:E14)</f>
-        <v>2.1091168362611213E+17</v>
+        <v>2.3780308157070598E+17</v>
       </c>
       <c r="F15" s="4">
         <f>AVERAGE(F2:F14)</f>
-        <v>1.7431053866382142E+24</v>
+        <v>1.9521791325723204E+24</v>
       </c>
       <c r="G15" s="1"/>
     </row>
@@ -1132,7 +1134,7 @@
       <c r="C16" s="1"/>
       <c r="F16" s="5">
         <f>_xlfn.STDEV.P(F2:F14)</f>
-        <v>6.5231872031064794E+23</v>
+        <v>6.9264413405437013E+23</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1141,8 +1143,11 @@
       </c>
       <c r="F17" s="6">
         <f>(F16/F15)</f>
-        <v>0.37422792982627523</v>
-      </c>
+        <v>0.35480562336597482</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D23" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1187,17 +1192,20 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>7.7764194500502032E+16</v>
+        <v>9.8997519685212848E+16</v>
       </c>
       <c r="C2">
-        <v>5.3690535730283398E+23</v>
+        <v>6.806128774716576E+23</v>
       </c>
       <c r="D2">
-        <v>6904274.656884254</v>
+        <v>6875049.7955487669</v>
+      </c>
+      <c r="E2">
+        <v>9.9254718252437792E+16</v>
       </c>
       <c r="F2">
         <f>D2*E2</f>
-        <v>0</v>
+        <v>6.8238113042867285E+23</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1205,17 +1213,20 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>7.6198879250466976E+16</v>
+        <v>9.7054047710008816E+16</v>
       </c>
       <c r="C3">
-        <v>1.023039500383313E+24</v>
+        <v>1.3119701329388659E+24</v>
       </c>
       <c r="D3">
-        <v>13425912.6964396</v>
+        <v>13517933.19181234</v>
+      </c>
+      <c r="E3">
+        <v>9.8349139155167872E+16</v>
       </c>
       <c r="F3">
         <f t="shared" ref="F3:F14" si="0">D3*E3</f>
-        <v>0</v>
+        <v>1.3294770925718143E+24</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1223,17 +1234,20 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>7.7764194500502032E+16</v>
+        <v>9.8997519685212848E+16</v>
       </c>
       <c r="C4">
-        <v>8.2465463014404721E+23</v>
+        <v>1.048452848425199E+24</v>
       </c>
       <c r="D4">
-        <v>10604554.389600519</v>
+        <v>10590698.14838811</v>
+      </c>
+      <c r="E4">
+        <v>9.9254718252437792E+16</v>
       </c>
       <c r="F4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.0511767608148764E+24</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1241,17 +1255,20 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>7.7748868259803664E+16</v>
+        <v>9.8978659271422608E+16</v>
       </c>
       <c r="C5">
-        <v>9.1014496617285321E+23</v>
+        <v>1.1605487584760041E+24</v>
       </c>
       <c r="D5">
-        <v>11706214.978352301</v>
+        <v>11725242.259480489</v>
+      </c>
+      <c r="E5">
+        <v>9.9254716400402048E+16</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.1637855951907453E+24</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1259,17 +1276,20 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>7.376957628198312E+16</v>
+        <v>1.0520607946173501E+17</v>
       </c>
       <c r="C6">
-        <v>5.0491714788632579E+23</v>
+        <v>7.1255366489034392E+23</v>
       </c>
       <c r="D6">
-        <v>6844517.3923229193</v>
+        <v>6772932.4059595829</v>
+      </c>
+      <c r="E6">
+        <v>1.0718470454866781E+17</v>
       </c>
       <c r="F6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.259547588608757E+23</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1277,17 +1297,20 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>7.5491866446378448E+16</v>
+        <v>9.692188295975464E+16</v>
       </c>
       <c r="C7">
-        <v>5.9367410286852901E+23</v>
+        <v>7.546419656966663E+23</v>
       </c>
       <c r="D7">
-        <v>7864080.3415585598</v>
+        <v>7786084.4491642835</v>
+      </c>
+      <c r="E7">
+        <v>9.816586382952376E+16</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.6432770580183354E+23</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1295,17 +1318,20 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>6.2102467643042152E+16</v>
+        <v>9.8306230172299728E+16</v>
       </c>
       <c r="C8">
-        <v>2.6367730155851471E+23</v>
+        <v>4.0577997622483843E+23</v>
       </c>
       <c r="D8">
-        <v>4245842.5818777699</v>
+        <v>4127713.7320150961</v>
+      </c>
+      <c r="E8">
+        <v>9.8917608776541024E+16</v>
       </c>
       <c r="F8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.0830357208502536E+23</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1313,17 +1339,20 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>3.2130549322872512E+16</v>
+        <v>8.4868446225645136E+16</v>
       </c>
       <c r="C9">
-        <v>2.4075230656500088E+23</v>
+        <v>6.3591425026981582E+23</v>
       </c>
       <c r="D9">
-        <v>7492940.8814563435</v>
+        <v>7492940.8814563444</v>
+      </c>
+      <c r="E9">
+        <v>8.5136012401282288E+16</v>
       </c>
       <c r="F9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.3791910780574239E+23</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1331,17 +1360,20 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>7.660576141561976E+16</v>
+        <v>9.831532867640984E+16</v>
       </c>
       <c r="C10">
-        <v>9.4266038085827665E+23</v>
+        <v>1.200748845507542E+24</v>
       </c>
       <c r="D10">
-        <v>12305345.752572469</v>
+        <v>12213241.431146789</v>
+      </c>
+      <c r="E10">
+        <v>9.831532867640984E+16</v>
       </c>
       <c r="F10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.2007488455075427E+24</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1349,17 +1381,20 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>7.6038809139919296E+16</v>
+        <v>9.7624974260697472E+16</v>
       </c>
       <c r="C11">
-        <v>4.8842658163226999E+23</v>
+        <v>6.3135341292384631E+23</v>
       </c>
       <c r="D11">
-        <v>6423385.46798536</v>
+        <v>6467130.1345276861</v>
+      </c>
+      <c r="E11">
+        <v>9.7637103414883072E+16</v>
       </c>
       <c r="F11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.3143185374238632E+23</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1367,17 +1402,20 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>5.7668476635642736E+16</v>
+        <v>9.530807071650264E+16</v>
       </c>
       <c r="C12">
-        <v>4.1818618610380989E+23</v>
+        <v>6.9128380329750863E+23</v>
       </c>
       <c r="D12">
-        <v>7251555.9713145709</v>
+        <v>7253150.7363501014</v>
+      </c>
+      <c r="E12">
+        <v>9.6085618216996032E+16</v>
       </c>
       <c r="F12">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.9692347252325951E+23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1385,17 +1423,20 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>7.841357058805848E+16</v>
+        <v>9.3995701884305488E+16</v>
       </c>
       <c r="C13">
-        <v>3.5644966160858241E+23</v>
+        <v>4.3475246096016561E+23</v>
       </c>
       <c r="D13">
-        <v>4545764.9605215881</v>
+        <v>4625237.6677316613</v>
+      </c>
+      <c r="E13">
+        <v>9.3995701884305488E+16</v>
       </c>
       <c r="F13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.3475246096016561E+23</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1403,17 +1444,20 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>8.0684046363406064E+16</v>
+        <v>9.66847035757388E+16</v>
       </c>
       <c r="C14">
-        <v>3.617533126784654E+23</v>
+        <v>4.3384105191578622E+23</v>
       </c>
       <c r="D14">
-        <v>4483579.2078288384</v>
+        <v>4487173.6259286664</v>
+      </c>
+      <c r="E14">
+        <v>9.66847035757388E+16</v>
       </c>
       <c r="F14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.3384105191578615E+23</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1422,23 +1466,23 @@
       </c>
       <c r="B15" s="2">
         <f>AVERAGE(B2:B14)</f>
-        <v>7.0952404642169032E+16</v>
+        <v>9.7019935714226608E+16</v>
       </c>
       <c r="C15" s="2">
         <f t="shared" ref="C15:F15" si="1">AVERAGE(C2:C14)</f>
-        <v>5.7424934121252486E+23</v>
+        <v>7.7711184992294152E+23</v>
       </c>
       <c r="D15" s="2">
         <f t="shared" si="1"/>
-        <v>8007536.0983626992</v>
-      </c>
-      <c r="E15" s="2" t="e">
+        <v>7994963.727654608</v>
+      </c>
+      <c r="E15" s="2">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>9.755661056806104E+16</v>
       </c>
       <c r="F15" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7.8161718524682517E+23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add refined data files for CESM2
</commit_message>
<xml_diff>
--- a/Data/OHC_diff_totals_output_glob.xlsx
+++ b/Data/OHC_diff_totals_output_glob.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harry\01.HarryGrosvenor\02.Research\05.Local_Repos\202404_01.PlioMIP2_ThetaO\Data\01.thetao\01.OneTime\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95D335E4-8D19-4A1D-A562-18F993A836C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DB5CDD-0D46-402A-A63B-47AC6122A1F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9000" yWindow="12852" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4395" yWindow="2430" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OHC diffs Globally" sheetId="1" r:id="rId1"/>
@@ -557,21 +557,21 @@
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>1.313275627826538E+18</v>
       </c>
-      <c r="C5" s="3">
-        <v>1.3128851875734359E+25</v>
-      </c>
-      <c r="D5" s="3">
-        <v>9997026.9740423933</v>
+      <c r="C5">
+        <v>1.5457580029379809E+25</v>
+      </c>
+      <c r="D5">
+        <v>11770248.1503917</v>
       </c>
       <c r="E5" s="3">
         <v>1.3252998821679491E+18</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>1.3249058670728193E+25</v>
+        <v>1.5599108486801639E+25</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -773,11 +773,11 @@
       </c>
       <c r="C15" s="4">
         <f t="shared" ref="C15:F15" si="1">AVERAGE(C2:C14)</f>
-        <v>8.8768004978927817E+24</v>
+        <v>9.0559334327885867E+24</v>
       </c>
       <c r="D15" s="4">
         <f t="shared" si="1"/>
-        <v>7524846.9505894026</v>
+        <v>7661248.5795393493</v>
       </c>
       <c r="E15" s="4">
         <f>AVERAGE(E2:E14)</f>
@@ -785,7 +785,7 @@
       </c>
       <c r="F15" s="4">
         <f t="shared" si="1"/>
-        <v>9.0403258876127506E+24</v>
+        <v>9.2210989503876309E+24</v>
       </c>
     </row>
   </sheetData>
@@ -894,21 +894,21 @@
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5">
         <v>2.3980392349821709E+17</v>
       </c>
-      <c r="C5" s="3">
-        <v>2.7873187196668302E+24</v>
-      </c>
-      <c r="D5" s="3">
-        <v>11623324.084968749</v>
+      <c r="C5">
+        <v>3.023216057751153E+24</v>
+      </c>
+      <c r="D5">
+        <v>12607033.33644009</v>
       </c>
       <c r="E5">
         <v>2.413631143030385E+17</v>
       </c>
       <c r="F5" s="7">
         <f t="shared" si="0"/>
-        <v>2.8054416997015724E+24</v>
+        <v>3.0428728282054061E+24</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1111,11 +1111,11 @@
       </c>
       <c r="C15" s="4">
         <f>AVERAGE(C2:C14)</f>
-        <v>1.9351144001694285E+24</v>
+        <v>1.9532603492528379E+24</v>
       </c>
       <c r="D15" s="4">
         <f>AVERAGE(D2:D14)</f>
-        <v>8189129.093910858</v>
+        <v>8264799.03633173</v>
       </c>
       <c r="E15" s="4">
         <f>AVERAGE(E2:E14)</f>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="F15" s="4">
         <f>AVERAGE(F2:F14)</f>
-        <v>1.9521791325723204E+24</v>
+        <v>1.9704430655341539E+24</v>
       </c>
       <c r="G15" s="1"/>
     </row>
@@ -1134,7 +1134,7 @@
       <c r="C16" s="1"/>
       <c r="F16" s="5">
         <f>_xlfn.STDEV.P(F2:F14)</f>
-        <v>6.9264413405437013E+23</v>
+        <v>7.1758387109558218E+23</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F17" s="6">
         <f>(F16/F15)</f>
-        <v>0.35480562336597482</v>
+        <v>0.36417386710996252</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1258,17 +1258,17 @@
         <v>9.8978659271422608E+16</v>
       </c>
       <c r="C5">
-        <v>1.1605487584760041E+24</v>
+        <v>1.2625838177244569E+24</v>
       </c>
       <c r="D5">
-        <v>11725242.259480489</v>
+        <v>12756121.64297111</v>
       </c>
       <c r="E5">
         <v>9.9254716400402048E+16</v>
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>1.1637855951907453E+24</v>
+        <v>1.2661052360421282E+24</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1470,11 +1470,11 @@
       </c>
       <c r="C15" s="2">
         <f t="shared" ref="C15:F15" si="1">AVERAGE(C2:C14)</f>
-        <v>7.7711184992294152E+23</v>
+        <v>7.849607006343609E+23</v>
       </c>
       <c r="D15" s="2">
         <f t="shared" si="1"/>
-        <v>7994963.727654608</v>
+        <v>8074262.1417692713</v>
       </c>
       <c r="E15" s="2">
         <f t="shared" si="1"/>
@@ -1482,7 +1482,7 @@
       </c>
       <c r="F15" s="2">
         <f t="shared" si="1"/>
-        <v>7.8161718524682517E+23</v>
+        <v>7.8948792685077758E+23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>